<commit_message>
Merge detailed Winter 2027 registration rules into target_courses
- sections.json/csv: additive registration_* fields (structured rules, notes,
  source URLs) for 90 of 115 sections across CSE 311/312/331/332/351/373 and
  AMATH 301/351/352/482; all original fields unchanged
- Add registration_rules.json (consolidated evidence) and REGISTRATION_MERGE.md
- Update README, metadata (v3) and workbook; point metadata at
  data/handoff/winter_2027_registration_review.json
- Re-pin sections.json SHA-256 in registration_evidence_handoff.json
- projected_offerings.json kept (not part of the data drop)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/target_courses/UniFlow_Winter_2027.xlsx
+++ b/data/target_courses/UniFlow_Winter_2027.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Courses" sheetId="1" r:id="R8f265768e68e4d6b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sections" sheetId="2" r:id="Re3159a0516b74420"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prerequisites" sheetId="3" r:id="Rd1b8012c3698449b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Courses" sheetId="1" r:id="R7d30eba9c0644321"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sections" sheetId="2" r:id="R7a432ecdeb2c4195"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prerequisites" sheetId="3" r:id="R17bb3966582f40f0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -42,12 +42,17 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="5">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF352A57"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -66,7 +71,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="23">
+  <x:cellXfs count="29">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -132,6 +137,24 @@
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -162,7 +185,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF1CC"/>
         </x:patternFill>
       </x:fill>
@@ -197,8 +220,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="SectionsData" displayName="SectionsData" ref="A1:U116" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="21">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="SectionsData" displayName="SectionsData" ref="A1:AA116" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="27">
     <x:tableColumn id="1" name="course_id"/>
     <x:tableColumn id="2" name="term"/>
     <x:tableColumn id="3" name="section"/>
@@ -220,6 +243,12 @@
     <x:tableColumn id="19" name="source_url"/>
     <x:tableColumn id="20" name="detail_url"/>
     <x:tableColumn id="21" name="snapshot_at"/>
+    <x:tableColumn id="22" name="registration_detail_status"/>
+    <x:tableColumn id="23" name="registration_status"/>
+    <x:tableColumn id="24" name="registration_rules_summary"/>
+    <x:tableColumn id="25" name="registration_notes"/>
+    <x:tableColumn id="26" name="registration_source_url"/>
+    <x:tableColumn id="27" name="registration_checked_at"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -3803,7 +3832,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12c823433cb04968"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R783dcd2562684172"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3833,6 +3862,12 @@
     <x:col min="19" max="19" width="70" hidden="0" customWidth="1"/>
     <x:col min="20" max="20" width="70" hidden="0" customWidth="1"/>
     <x:col min="21" max="21" width="25" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="28" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="22" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="82" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="84" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="80" hidden="0" customWidth="1"/>
+    <x:col min="27" max="27" width="25" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
@@ -3899,8 +3934,26 @@
       <x:c r="U1" s="14" t="str">
         <x:v>snapshot_at</x:v>
       </x:c>
-    </x:row>
-    <x:row r="2" ht="60" customHeight="1">
+      <x:c r="V1" s="28" t="str">
+        <x:v>registration_detail_status</x:v>
+      </x:c>
+      <x:c r="W1" s="28" t="str">
+        <x:v>registration_status</x:v>
+      </x:c>
+      <x:c r="X1" s="28" t="str">
+        <x:v>registration_rules_summary</x:v>
+      </x:c>
+      <x:c r="Y1" s="28" t="str">
+        <x:v>registration_notes</x:v>
+      </x:c>
+      <x:c r="Z1" s="28" t="str">
+        <x:v>registration_source_url</x:v>
+      </x:c>
+      <x:c r="AA1" s="28" t="str">
+        <x:v>registration_checked_at</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="108" customHeight="1">
       <x:c r="A2" s="3" t="str">
         <x:v>CSE 311</x:v>
       </x:c>
@@ -3960,8 +4013,32 @@
       <x:c r="U2" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="3" ht="60" customHeight="1">
+      <x:c r="V2" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W2" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X2" s="23" t="str">
+        <x:v>Majors only: C SCI, CMP E</x:v>
+      </x:c>
+      <x:c r="Y2" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+C SCI,CMP E majors only
+--
+FINAL EXAM TENTATIVELY PLANNED FOR
+MARCH 15, 1230-220PM
+--</x:v>
+      </x:c>
+      <x:c r="Z2" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12854</x:v>
+      </x:c>
+      <x:c r="AA2" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="80" customHeight="1">
       <x:c r="A3" s="3" t="str">
         <x:v>CSE 311</x:v>
       </x:c>
@@ -4015,8 +4092,28 @@
       <x:c r="U3" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="4" ht="60" customHeight="1">
+      <x:c r="V3" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W3" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X3" s="23" t="str">
+        <x:v>No additional structured restriction in captured Notes. Full eligibility remains unknown.</x:v>
+      </x:c>
+      <x:c r="Y3" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z3" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12855</x:v>
+      </x:c>
+      <x:c r="AA3" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="80" customHeight="1">
       <x:c r="A4" s="3" t="str">
         <x:v>CSE 311</x:v>
       </x:c>
@@ -4070,8 +4167,28 @@
       <x:c r="U4" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="5" ht="60" customHeight="1">
+      <x:c r="V4" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W4" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X4" s="23" t="str">
+        <x:v>No additional structured restriction in captured Notes. Full eligibility remains unknown.</x:v>
+      </x:c>
+      <x:c r="Y4" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z4" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12856</x:v>
+      </x:c>
+      <x:c r="AA4" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="80" customHeight="1">
       <x:c r="A5" s="3" t="str">
         <x:v>CSE 311</x:v>
       </x:c>
@@ -4125,8 +4242,28 @@
       <x:c r="U5" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="6" ht="60" customHeight="1">
+      <x:c r="V5" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W5" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X5" s="23" t="str">
+        <x:v>No additional structured restriction in captured Notes. Full eligibility remains unknown.</x:v>
+      </x:c>
+      <x:c r="Y5" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z5" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12857</x:v>
+      </x:c>
+      <x:c r="AA5" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="80" customHeight="1">
       <x:c r="A6" s="3" t="str">
         <x:v>CSE 311</x:v>
       </x:c>
@@ -4180,8 +4317,28 @@
       <x:c r="U6" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="7" ht="60" customHeight="1">
+      <x:c r="V6" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W6" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X6" s="23" t="str">
+        <x:v>No additional structured restriction in captured Notes. Full eligibility remains unknown.</x:v>
+      </x:c>
+      <x:c r="Y6" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z6" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12858</x:v>
+      </x:c>
+      <x:c r="AA6" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="80" customHeight="1">
       <x:c r="A7" s="3" t="str">
         <x:v>CSE 311</x:v>
       </x:c>
@@ -4235,8 +4392,28 @@
       <x:c r="U7" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="8" ht="60" customHeight="1">
+      <x:c r="V7" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W7" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X7" s="23" t="str">
+        <x:v>No additional structured restriction in captured Notes. Full eligibility remains unknown.</x:v>
+      </x:c>
+      <x:c r="Y7" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z7" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12859</x:v>
+      </x:c>
+      <x:c r="AA7" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="108" customHeight="1">
       <x:c r="A8" s="3" t="str">
         <x:v>CSE 311</x:v>
       </x:c>
@@ -4296,8 +4473,32 @@
       <x:c r="U8" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="9" ht="60" customHeight="1">
+      <x:c r="V8" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W8" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X8" s="23" t="str">
+        <x:v>Majors only: C SCI, CMP E</x:v>
+      </x:c>
+      <x:c r="Y8" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+C SCI,CMP E majors only
+--
+FINAL EXAM TENTATIVELY PLANNED FOR
+MARCH 15, 1230-220PM
+--</x:v>
+      </x:c>
+      <x:c r="Z8" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12860</x:v>
+      </x:c>
+      <x:c r="AA8" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="80" customHeight="1">
       <x:c r="A9" s="3" t="str">
         <x:v>CSE 311</x:v>
       </x:c>
@@ -4351,8 +4552,28 @@
       <x:c r="U9" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="10" ht="60" customHeight="1">
+      <x:c r="V9" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W9" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X9" s="23" t="str">
+        <x:v>No additional structured restriction in captured Notes. Full eligibility remains unknown.</x:v>
+      </x:c>
+      <x:c r="Y9" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z9" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12861</x:v>
+      </x:c>
+      <x:c r="AA9" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="80" customHeight="1">
       <x:c r="A10" s="3" t="str">
         <x:v>CSE 311</x:v>
       </x:c>
@@ -4406,8 +4627,28 @@
       <x:c r="U10" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="11" ht="60" customHeight="1">
+      <x:c r="V10" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W10" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X10" s="23" t="str">
+        <x:v>No additional structured restriction in captured Notes. Full eligibility remains unknown.</x:v>
+      </x:c>
+      <x:c r="Y10" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z10" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12862</x:v>
+      </x:c>
+      <x:c r="AA10" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="80" customHeight="1">
       <x:c r="A11" s="3" t="str">
         <x:v>CSE 311</x:v>
       </x:c>
@@ -4461,8 +4702,28 @@
       <x:c r="U11" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="12" ht="60" customHeight="1">
+      <x:c r="V11" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W11" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X11" s="23" t="str">
+        <x:v>No additional structured restriction in captured Notes. Full eligibility remains unknown.</x:v>
+      </x:c>
+      <x:c r="Y11" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z11" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12863</x:v>
+      </x:c>
+      <x:c r="AA11" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="80" customHeight="1">
       <x:c r="A12" s="3" t="str">
         <x:v>CSE 311</x:v>
       </x:c>
@@ -4516,8 +4777,28 @@
       <x:c r="U12" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="13" ht="60" customHeight="1">
+      <x:c r="V12" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W12" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X12" s="23" t="str">
+        <x:v>No additional structured restriction in captured Notes. Full eligibility remains unknown.</x:v>
+      </x:c>
+      <x:c r="Y12" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z12" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12864</x:v>
+      </x:c>
+      <x:c r="AA12" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="80" customHeight="1">
       <x:c r="A13" s="3" t="str">
         <x:v>CSE 311</x:v>
       </x:c>
@@ -4571,8 +4852,28 @@
       <x:c r="U13" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="14" ht="60" customHeight="1">
+      <x:c r="V13" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W13" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X13" s="23" t="str">
+        <x:v>No additional structured restriction in captured Notes. Full eligibility remains unknown.</x:v>
+      </x:c>
+      <x:c r="Y13" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z13" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12865</x:v>
+      </x:c>
+      <x:c r="AA13" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="108" customHeight="1">
       <x:c r="A14" s="3" t="str">
         <x:v>CSE 312</x:v>
       </x:c>
@@ -4632,8 +4933,32 @@
       <x:c r="U14" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="15" ht="60" customHeight="1">
+      <x:c r="V14" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W14" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X14" s="23" t="str">
+        <x:v>Majors only: C SCI, CMP E</x:v>
+      </x:c>
+      <x:c r="Y14" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+C SCI,CMP E majors only
+--
+FINAL EXAM TENTATIVELY PLANNED FOR
+MARCH 15, 1230-220PM
+--</x:v>
+      </x:c>
+      <x:c r="Z14" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12866</x:v>
+      </x:c>
+      <x:c r="AA14" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="80" customHeight="1">
       <x:c r="A15" s="3" t="str">
         <x:v>CSE 312</x:v>
       </x:c>
@@ -4687,8 +5012,28 @@
       <x:c r="U15" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="16" ht="60" customHeight="1">
+      <x:c r="V15" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W15" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X15" s="23" t="str">
+        <x:v>No additional structured restriction in captured Notes. Full eligibility remains unknown.</x:v>
+      </x:c>
+      <x:c r="Y15" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z15" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12867</x:v>
+      </x:c>
+      <x:c r="AA15" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="80" customHeight="1">
       <x:c r="A16" s="3" t="str">
         <x:v>CSE 312</x:v>
       </x:c>
@@ -4742,8 +5087,28 @@
       <x:c r="U16" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="17" ht="60" customHeight="1">
+      <x:c r="V16" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W16" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X16" s="23" t="str">
+        <x:v>No additional structured restriction in captured Notes. Full eligibility remains unknown.</x:v>
+      </x:c>
+      <x:c r="Y16" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z16" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12868</x:v>
+      </x:c>
+      <x:c r="AA16" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="80" customHeight="1">
       <x:c r="A17" s="3" t="str">
         <x:v>CSE 312</x:v>
       </x:c>
@@ -4797,8 +5162,28 @@
       <x:c r="U17" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="18" ht="60" customHeight="1">
+      <x:c r="V17" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W17" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X17" s="23" t="str">
+        <x:v>No additional structured restriction in captured Notes. Full eligibility remains unknown.</x:v>
+      </x:c>
+      <x:c r="Y17" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z17" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12869</x:v>
+      </x:c>
+      <x:c r="AA17" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="80" customHeight="1">
       <x:c r="A18" s="3" t="str">
         <x:v>CSE 312</x:v>
       </x:c>
@@ -4852,8 +5237,28 @@
       <x:c r="U18" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="19" ht="60" customHeight="1">
+      <x:c r="V18" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W18" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X18" s="23" t="str">
+        <x:v>No additional structured restriction in captured Notes. Full eligibility remains unknown.</x:v>
+      </x:c>
+      <x:c r="Y18" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z18" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12870</x:v>
+      </x:c>
+      <x:c r="AA18" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="80" customHeight="1">
       <x:c r="A19" s="3" t="str">
         <x:v>CSE 312</x:v>
       </x:c>
@@ -4907,8 +5312,28 @@
       <x:c r="U19" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="20" ht="60" customHeight="1">
+      <x:c r="V19" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W19" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X19" s="23" t="str">
+        <x:v>No additional structured restriction in captured Notes. Full eligibility remains unknown.</x:v>
+      </x:c>
+      <x:c r="Y19" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z19" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12871</x:v>
+      </x:c>
+      <x:c r="AA19" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="108" customHeight="1">
       <x:c r="A20" s="3" t="str">
         <x:v>CSE 312</x:v>
       </x:c>
@@ -4966,8 +5391,32 @@
       <x:c r="U20" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="21" ht="60" customHeight="1">
+      <x:c r="V20" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W20" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X20" s="23" t="str">
+        <x:v>Joint offering: CSE 312 BF (SLN 12879). Not a lecture/quiz pairing approval</x:v>
+      </x:c>
+      <x:c r="Y20" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Offered jointly with CSE 312 BF
+Quiz Section
+--
+OPEN FOR REGISTRATION
+--</x:v>
+      </x:c>
+      <x:c r="Z20" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12872</x:v>
+      </x:c>
+      <x:c r="AA20" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="108" customHeight="1">
       <x:c r="A21" s="3" t="str">
         <x:v>CSE 312</x:v>
       </x:c>
@@ -5027,8 +5476,32 @@
       <x:c r="U21" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="22" ht="60" customHeight="1">
+      <x:c r="V21" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W21" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X21" s="23" t="str">
+        <x:v>Majors only: C SCI, CMP E</x:v>
+      </x:c>
+      <x:c r="Y21" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+C SCI,CMP E majors only
+--
+FINAL EXAM TENTATIVELY PLANNED FOR
+MARCH 15, 1230-220PM
+--</x:v>
+      </x:c>
+      <x:c r="Z21" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12873</x:v>
+      </x:c>
+      <x:c r="AA21" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="80" customHeight="1">
       <x:c r="A22" s="3" t="str">
         <x:v>CSE 312</x:v>
       </x:c>
@@ -5084,8 +5557,29 @@
       <x:c r="U22" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="23" ht="60" customHeight="1">
+      <x:c r="V22" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W22" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X22" s="23" t="str">
+        <x:v>Majors only: C SCI, CMP E</x:v>
+      </x:c>
+      <x:c r="Y22" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section
+C SCI,CMP E majors only</x:v>
+      </x:c>
+      <x:c r="Z22" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12874</x:v>
+      </x:c>
+      <x:c r="AA22" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="80" customHeight="1">
       <x:c r="A23" s="3" t="str">
         <x:v>CSE 312</x:v>
       </x:c>
@@ -5141,8 +5635,29 @@
       <x:c r="U23" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="24" ht="60" customHeight="1">
+      <x:c r="V23" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W23" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X23" s="23" t="str">
+        <x:v>Majors only: C SCI, CMP E</x:v>
+      </x:c>
+      <x:c r="Y23" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section
+C SCI,CMP E majors only</x:v>
+      </x:c>
+      <x:c r="Z23" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12875</x:v>
+      </x:c>
+      <x:c r="AA23" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="80" customHeight="1">
       <x:c r="A24" s="3" t="str">
         <x:v>CSE 312</x:v>
       </x:c>
@@ -5198,8 +5713,29 @@
       <x:c r="U24" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="25" ht="60" customHeight="1">
+      <x:c r="V24" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W24" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X24" s="23" t="str">
+        <x:v>Majors only: C SCI, CMP E</x:v>
+      </x:c>
+      <x:c r="Y24" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section
+C SCI,CMP E majors only</x:v>
+      </x:c>
+      <x:c r="Z24" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12876</x:v>
+      </x:c>
+      <x:c r="AA24" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="80" customHeight="1">
       <x:c r="A25" s="3" t="str">
         <x:v>CSE 312</x:v>
       </x:c>
@@ -5255,8 +5791,29 @@
       <x:c r="U25" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="26" ht="60" customHeight="1">
+      <x:c r="V25" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W25" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X25" s="23" t="str">
+        <x:v>Majors only: C SCI, CMP E</x:v>
+      </x:c>
+      <x:c r="Y25" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section
+C SCI,CMP E majors only</x:v>
+      </x:c>
+      <x:c r="Z25" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12877</x:v>
+      </x:c>
+      <x:c r="AA25" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="80" customHeight="1">
       <x:c r="A26" s="3" t="str">
         <x:v>CSE 312</x:v>
       </x:c>
@@ -5312,8 +5869,29 @@
       <x:c r="U26" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="27" ht="60" customHeight="1">
+      <x:c r="V26" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W26" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X26" s="23" t="str">
+        <x:v>Majors only: C SCI, CMP E</x:v>
+      </x:c>
+      <x:c r="Y26" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section
+C SCI,CMP E majors only</x:v>
+      </x:c>
+      <x:c r="Z26" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12878</x:v>
+      </x:c>
+      <x:c r="AA26" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="122" customHeight="1">
       <x:c r="A27" s="3" t="str">
         <x:v>CSE 312</x:v>
       </x:c>
@@ -5373,8 +5951,34 @@
       <x:c r="U27" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="28" ht="60" customHeight="1">
+      <x:c r="V27" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W27" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X27" s="23" t="str">
+        <x:v>Joint offering: CSE 312 AF (SLN 12872). Not a lecture/quiz pairing approval
+Majors only: C SCI, CMP E</x:v>
+      </x:c>
+      <x:c r="Y27" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Offered jointly with CSE 312 AF
+Quiz Section
+C SCI,CMP E majors only
+--
+OPEN FOR REGISTRATION
+--</x:v>
+      </x:c>
+      <x:c r="Z27" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12879</x:v>
+      </x:c>
+      <x:c r="AA27" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="108" customHeight="1">
       <x:c r="A28" s="3" t="str">
         <x:v>CSE 331</x:v>
       </x:c>
@@ -5434,8 +6038,32 @@
       <x:c r="U28" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="29" ht="60" customHeight="1">
+      <x:c r="V28" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W28" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X28" s="23" t="str">
+        <x:v>Majors only: C SCI, CMP E</x:v>
+      </x:c>
+      <x:c r="Y28" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+C SCI,CMP E majors only
+--
+FINAL EXAM TENTATIVELY PLANNED FOR
+MARCH 16, 1230-220PM
+--</x:v>
+      </x:c>
+      <x:c r="Z28" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12880</x:v>
+      </x:c>
+      <x:c r="AA28" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="80" customHeight="1">
       <x:c r="A29" s="3" t="str">
         <x:v>CSE 331</x:v>
       </x:c>
@@ -5489,8 +6117,28 @@
       <x:c r="U29" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="30" ht="60" customHeight="1">
+      <x:c r="V29" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W29" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X29" s="23" t="str">
+        <x:v>No additional structured restriction in captured Notes. Full eligibility remains unknown.</x:v>
+      </x:c>
+      <x:c r="Y29" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z29" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12881</x:v>
+      </x:c>
+      <x:c r="AA29" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="80" customHeight="1">
       <x:c r="A30" s="3" t="str">
         <x:v>CSE 331</x:v>
       </x:c>
@@ -5544,8 +6192,28 @@
       <x:c r="U30" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="31" ht="60" customHeight="1">
+      <x:c r="V30" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W30" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X30" s="23" t="str">
+        <x:v>No additional structured restriction in captured Notes. Full eligibility remains unknown.</x:v>
+      </x:c>
+      <x:c r="Y30" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z30" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12882</x:v>
+      </x:c>
+      <x:c r="AA30" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="80" customHeight="1">
       <x:c r="A31" s="3" t="str">
         <x:v>CSE 331</x:v>
       </x:c>
@@ -5599,8 +6267,28 @@
       <x:c r="U31" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="32" ht="60" customHeight="1">
+      <x:c r="V31" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W31" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X31" s="23" t="str">
+        <x:v>No additional structured restriction in captured Notes. Full eligibility remains unknown.</x:v>
+      </x:c>
+      <x:c r="Y31" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z31" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12883</x:v>
+      </x:c>
+      <x:c r="AA31" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="80" customHeight="1">
       <x:c r="A32" s="3" t="str">
         <x:v>CSE 331</x:v>
       </x:c>
@@ -5654,8 +6342,28 @@
       <x:c r="U32" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="33" ht="60" customHeight="1">
+      <x:c r="V32" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W32" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X32" s="23" t="str">
+        <x:v>No additional structured restriction in captured Notes. Full eligibility remains unknown.</x:v>
+      </x:c>
+      <x:c r="Y32" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z32" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12884</x:v>
+      </x:c>
+      <x:c r="AA32" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="108" customHeight="1">
       <x:c r="A33" s="3" t="str">
         <x:v>CSE 331</x:v>
       </x:c>
@@ -5715,8 +6423,32 @@
       <x:c r="U33" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="34" ht="60" customHeight="1">
+      <x:c r="V33" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W33" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X33" s="23" t="str">
+        <x:v>Majors only: C SCI, CMP E</x:v>
+      </x:c>
+      <x:c r="Y33" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+C SCI,CMP E majors only
+--
+FINAL EXAM TENTATIVELY PLANNED FOR
+MARCH 16, 1230-220PM
+--</x:v>
+      </x:c>
+      <x:c r="Z33" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12885</x:v>
+      </x:c>
+      <x:c r="AA33" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="80" customHeight="1">
       <x:c r="A34" s="3" t="str">
         <x:v>CSE 331</x:v>
       </x:c>
@@ -5770,8 +6502,28 @@
       <x:c r="U34" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="35" ht="60" customHeight="1">
+      <x:c r="V34" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W34" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X34" s="23" t="str">
+        <x:v>No additional structured restriction in captured Notes. Full eligibility remains unknown.</x:v>
+      </x:c>
+      <x:c r="Y34" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z34" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12886</x:v>
+      </x:c>
+      <x:c r="AA34" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="80" customHeight="1">
       <x:c r="A35" s="3" t="str">
         <x:v>CSE 331</x:v>
       </x:c>
@@ -5825,8 +6577,28 @@
       <x:c r="U35" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="36" ht="60" customHeight="1">
+      <x:c r="V35" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W35" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X35" s="23" t="str">
+        <x:v>No additional structured restriction in captured Notes. Full eligibility remains unknown.</x:v>
+      </x:c>
+      <x:c r="Y35" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z35" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12887</x:v>
+      </x:c>
+      <x:c r="AA35" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="80" customHeight="1">
       <x:c r="A36" s="3" t="str">
         <x:v>CSE 331</x:v>
       </x:c>
@@ -5880,8 +6652,28 @@
       <x:c r="U36" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="37" ht="60" customHeight="1">
+      <x:c r="V36" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W36" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X36" s="23" t="str">
+        <x:v>No additional structured restriction in captured Notes. Full eligibility remains unknown.</x:v>
+      </x:c>
+      <x:c r="Y36" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z36" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12888</x:v>
+      </x:c>
+      <x:c r="AA36" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="80" customHeight="1">
       <x:c r="A37" s="3" t="str">
         <x:v>CSE 331</x:v>
       </x:c>
@@ -5935,8 +6727,28 @@
       <x:c r="U37" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="38" ht="60" customHeight="1">
+      <x:c r="V37" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W37" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X37" s="23" t="str">
+        <x:v>No additional structured restriction in captured Notes. Full eligibility remains unknown.</x:v>
+      </x:c>
+      <x:c r="Y37" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z37" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12889</x:v>
+      </x:c>
+      <x:c r="AA37" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="108" customHeight="1">
       <x:c r="A38" s="3" t="str">
         <x:v>CSE 332</x:v>
       </x:c>
@@ -5996,8 +6808,32 @@
       <x:c r="U38" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="39" ht="60" customHeight="1">
+      <x:c r="V38" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W38" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X38" s="23" t="str">
+        <x:v>Majors only: C SCI, CMP E</x:v>
+      </x:c>
+      <x:c r="Y38" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+C SCI,CMP E majors only
+--
+FINAL EXAM TENTATIVELY PLANNED FOR
+MARCH 18, 1230-220PM
+--</x:v>
+      </x:c>
+      <x:c r="Z38" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12890</x:v>
+      </x:c>
+      <x:c r="AA38" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="80" customHeight="1">
       <x:c r="A39" s="3" t="str">
         <x:v>CSE 332</x:v>
       </x:c>
@@ -6051,8 +6887,28 @@
       <x:c r="U39" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="40" ht="60" customHeight="1">
+      <x:c r="V39" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W39" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X39" s="23" t="str">
+        <x:v>No additional structured restriction in captured Notes. Full eligibility remains unknown.</x:v>
+      </x:c>
+      <x:c r="Y39" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z39" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12891</x:v>
+      </x:c>
+      <x:c r="AA39" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="80" customHeight="1">
       <x:c r="A40" s="3" t="str">
         <x:v>CSE 332</x:v>
       </x:c>
@@ -6106,8 +6962,28 @@
       <x:c r="U40" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="41" ht="60" customHeight="1">
+      <x:c r="V40" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W40" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X40" s="23" t="str">
+        <x:v>No additional structured restriction in captured Notes. Full eligibility remains unknown.</x:v>
+      </x:c>
+      <x:c r="Y40" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z40" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12892</x:v>
+      </x:c>
+      <x:c r="AA40" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="80" customHeight="1">
       <x:c r="A41" s="3" t="str">
         <x:v>CSE 332</x:v>
       </x:c>
@@ -6161,8 +7037,28 @@
       <x:c r="U41" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="42" ht="60" customHeight="1">
+      <x:c r="V41" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W41" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X41" s="23" t="str">
+        <x:v>No additional structured restriction in captured Notes. Full eligibility remains unknown.</x:v>
+      </x:c>
+      <x:c r="Y41" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z41" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12893</x:v>
+      </x:c>
+      <x:c r="AA41" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="80" customHeight="1">
       <x:c r="A42" s="3" t="str">
         <x:v>CSE 332</x:v>
       </x:c>
@@ -6216,8 +7112,28 @@
       <x:c r="U42" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="43" ht="60" customHeight="1">
+      <x:c r="V42" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W42" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X42" s="23" t="str">
+        <x:v>No additional structured restriction in captured Notes. Full eligibility remains unknown.</x:v>
+      </x:c>
+      <x:c r="Y42" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z42" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12894</x:v>
+      </x:c>
+      <x:c r="AA42" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="80" customHeight="1">
       <x:c r="A43" s="3" t="str">
         <x:v>CSE 332</x:v>
       </x:c>
@@ -6271,8 +7187,28 @@
       <x:c r="U43" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="44" ht="60" customHeight="1">
+      <x:c r="V43" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W43" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X43" s="23" t="str">
+        <x:v>No additional structured restriction in captured Notes. Full eligibility remains unknown.</x:v>
+      </x:c>
+      <x:c r="Y43" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z43" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12895</x:v>
+      </x:c>
+      <x:c r="AA43" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="80" customHeight="1">
       <x:c r="A44" s="3" t="str">
         <x:v>CSE 332</x:v>
       </x:c>
@@ -6330,8 +7266,30 @@
       <x:c r="U44" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="45" ht="60" customHeight="1">
+      <x:c r="V44" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W44" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X44" s="23" t="str">
+        <x:v>Joint offering: CSE 332 BD (SLN 12902). Not a lecture/quiz pairing approval</x:v>
+      </x:c>
+      <x:c r="Y44" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Offered jointly with CSE 332 BD
+Quiz Section
+AF/BD</x:v>
+      </x:c>
+      <x:c r="Z44" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12896</x:v>
+      </x:c>
+      <x:c r="AA44" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="80" customHeight="1">
       <x:c r="A45" s="3" t="str">
         <x:v>CSE 332</x:v>
       </x:c>
@@ -6385,8 +7343,28 @@
       <x:c r="U45" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="46" ht="60" customHeight="1">
+      <x:c r="V45" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W45" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X45" s="23" t="str">
+        <x:v>No additional structured restriction in captured Notes. Full eligibility remains unknown.</x:v>
+      </x:c>
+      <x:c r="Y45" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z45" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12897</x:v>
+      </x:c>
+      <x:c r="AA45" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="108" customHeight="1">
       <x:c r="A46" s="3" t="str">
         <x:v>CSE 332</x:v>
       </x:c>
@@ -6446,8 +7424,32 @@
       <x:c r="U46" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="47" ht="60" customHeight="1">
+      <x:c r="V46" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W46" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X46" s="23" t="str">
+        <x:v>Majors only: C SCI, CMP E</x:v>
+      </x:c>
+      <x:c r="Y46" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+C SCI,CMP E majors only
+--
+FINAL EXAM TENTATIVELY PLANNED FOR
+MARCH 18, 1230-220PM
+--</x:v>
+      </x:c>
+      <x:c r="Z46" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12898</x:v>
+      </x:c>
+      <x:c r="AA46" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="80" customHeight="1">
       <x:c r="A47" s="3" t="str">
         <x:v>CSE 332</x:v>
       </x:c>
@@ -6501,8 +7503,28 @@
       <x:c r="U47" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="48" ht="60" customHeight="1">
+      <x:c r="V47" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W47" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X47" s="23" t="str">
+        <x:v>No additional structured restriction in captured Notes. Full eligibility remains unknown.</x:v>
+      </x:c>
+      <x:c r="Y47" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z47" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12899</x:v>
+      </x:c>
+      <x:c r="AA47" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="80" customHeight="1">
       <x:c r="A48" s="3" t="str">
         <x:v>CSE 332</x:v>
       </x:c>
@@ -6556,8 +7578,28 @@
       <x:c r="U48" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="49" ht="60" customHeight="1">
+      <x:c r="V48" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W48" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X48" s="23" t="str">
+        <x:v>No additional structured restriction in captured Notes. Full eligibility remains unknown.</x:v>
+      </x:c>
+      <x:c r="Y48" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z48" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12900</x:v>
+      </x:c>
+      <x:c r="AA48" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="80" customHeight="1">
       <x:c r="A49" s="3" t="str">
         <x:v>CSE 332</x:v>
       </x:c>
@@ -6611,8 +7653,28 @@
       <x:c r="U49" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="50" ht="60" customHeight="1">
+      <x:c r="V49" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W49" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X49" s="23" t="str">
+        <x:v>No additional structured restriction in captured Notes. Full eligibility remains unknown.</x:v>
+      </x:c>
+      <x:c r="Y49" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z49" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12901</x:v>
+      </x:c>
+      <x:c r="AA49" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="80" customHeight="1">
       <x:c r="A50" s="3" t="str">
         <x:v>CSE 332</x:v>
       </x:c>
@@ -6669,6 +7731,28 @@
       </x:c>
       <x:c r="U50" s="11" t="n">
         <x:v>46312.00208333333</x:v>
+      </x:c>
+      <x:c r="V50" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W50" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X50" s="23" t="str">
+        <x:v>Joint offering: CSE 332 AF (SLN 12896). Not a lecture/quiz pairing approval</x:v>
+      </x:c>
+      <x:c r="Y50" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Offered jointly with CSE 332 AF
+Quiz Section
+AF/BD</x:v>
+      </x:c>
+      <x:c r="Z50" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12902</x:v>
+      </x:c>
+      <x:c r="AA50" s="24" t="n">
+        <x:v>46312.5</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="60" customHeight="1">
@@ -6729,6 +7813,12 @@
       <x:c r="U51" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
+      <x:c r="V51" s="23" t="str"/>
+      <x:c r="W51" s="23" t="str"/>
+      <x:c r="X51" s="23" t="str"/>
+      <x:c r="Y51" s="23" t="str"/>
+      <x:c r="Z51" s="23" t="str"/>
+      <x:c r="AA51" s="24" t="str"/>
     </x:row>
     <x:row r="52" ht="60" customHeight="1">
       <x:c r="A52" s="3" t="str">
@@ -6784,6 +7874,12 @@
       <x:c r="U52" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
+      <x:c r="V52" s="23" t="str"/>
+      <x:c r="W52" s="23" t="str"/>
+      <x:c r="X52" s="23" t="str"/>
+      <x:c r="Y52" s="23" t="str"/>
+      <x:c r="Z52" s="23" t="str"/>
+      <x:c r="AA52" s="24" t="str"/>
     </x:row>
     <x:row r="53" ht="60" customHeight="1">
       <x:c r="A53" s="3" t="str">
@@ -6839,6 +7935,12 @@
       <x:c r="U53" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
+      <x:c r="V53" s="23" t="str"/>
+      <x:c r="W53" s="23" t="str"/>
+      <x:c r="X53" s="23" t="str"/>
+      <x:c r="Y53" s="23" t="str"/>
+      <x:c r="Z53" s="23" t="str"/>
+      <x:c r="AA53" s="24" t="str"/>
     </x:row>
     <x:row r="54" ht="60" customHeight="1">
       <x:c r="A54" s="3" t="str">
@@ -6894,6 +7996,12 @@
       <x:c r="U54" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
+      <x:c r="V54" s="23" t="str"/>
+      <x:c r="W54" s="23" t="str"/>
+      <x:c r="X54" s="23" t="str"/>
+      <x:c r="Y54" s="23" t="str"/>
+      <x:c r="Z54" s="23" t="str"/>
+      <x:c r="AA54" s="24" t="str"/>
     </x:row>
     <x:row r="55" ht="60" customHeight="1">
       <x:c r="A55" s="3" t="str">
@@ -6949,6 +8057,12 @@
       <x:c r="U55" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
+      <x:c r="V55" s="23" t="str"/>
+      <x:c r="W55" s="23" t="str"/>
+      <x:c r="X55" s="23" t="str"/>
+      <x:c r="Y55" s="23" t="str"/>
+      <x:c r="Z55" s="23" t="str"/>
+      <x:c r="AA55" s="24" t="str"/>
     </x:row>
     <x:row r="56" ht="60" customHeight="1">
       <x:c r="A56" s="3" t="str">
@@ -7004,6 +8118,12 @@
       <x:c r="U56" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
+      <x:c r="V56" s="23" t="str"/>
+      <x:c r="W56" s="23" t="str"/>
+      <x:c r="X56" s="23" t="str"/>
+      <x:c r="Y56" s="23" t="str"/>
+      <x:c r="Z56" s="23" t="str"/>
+      <x:c r="AA56" s="24" t="str"/>
     </x:row>
     <x:row r="57" ht="60" customHeight="1">
       <x:c r="A57" s="3" t="str">
@@ -7061,6 +8181,12 @@
       <x:c r="U57" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
+      <x:c r="V57" s="23" t="str"/>
+      <x:c r="W57" s="23" t="str"/>
+      <x:c r="X57" s="23" t="str"/>
+      <x:c r="Y57" s="23" t="str"/>
+      <x:c r="Z57" s="23" t="str"/>
+      <x:c r="AA57" s="24" t="str"/>
     </x:row>
     <x:row r="58" ht="60" customHeight="1">
       <x:c r="A58" s="3" t="str">
@@ -7118,6 +8244,12 @@
       <x:c r="U58" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
+      <x:c r="V58" s="23" t="str"/>
+      <x:c r="W58" s="23" t="str"/>
+      <x:c r="X58" s="23" t="str"/>
+      <x:c r="Y58" s="23" t="str"/>
+      <x:c r="Z58" s="23" t="str"/>
+      <x:c r="AA58" s="24" t="str"/>
     </x:row>
     <x:row r="59" ht="60" customHeight="1">
       <x:c r="A59" s="3" t="str">
@@ -7177,6 +8309,12 @@
       <x:c r="U59" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
+      <x:c r="V59" s="23" t="str"/>
+      <x:c r="W59" s="23" t="str"/>
+      <x:c r="X59" s="23" t="str"/>
+      <x:c r="Y59" s="23" t="str"/>
+      <x:c r="Z59" s="23" t="str"/>
+      <x:c r="AA59" s="24" t="str"/>
     </x:row>
     <x:row r="60" ht="60" customHeight="1">
       <x:c r="A60" s="3" t="str">
@@ -7232,6 +8370,12 @@
       <x:c r="U60" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
+      <x:c r="V60" s="23" t="str"/>
+      <x:c r="W60" s="23" t="str"/>
+      <x:c r="X60" s="23" t="str"/>
+      <x:c r="Y60" s="23" t="str"/>
+      <x:c r="Z60" s="23" t="str"/>
+      <x:c r="AA60" s="24" t="str"/>
     </x:row>
     <x:row r="61" ht="60" customHeight="1">
       <x:c r="A61" s="3" t="str">
@@ -7287,6 +8431,12 @@
       <x:c r="U61" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
+      <x:c r="V61" s="23" t="str"/>
+      <x:c r="W61" s="23" t="str"/>
+      <x:c r="X61" s="23" t="str"/>
+      <x:c r="Y61" s="23" t="str"/>
+      <x:c r="Z61" s="23" t="str"/>
+      <x:c r="AA61" s="24" t="str"/>
     </x:row>
     <x:row r="62" ht="60" customHeight="1">
       <x:c r="A62" s="3" t="str">
@@ -7342,6 +8492,12 @@
       <x:c r="U62" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
+      <x:c r="V62" s="23" t="str"/>
+      <x:c r="W62" s="23" t="str"/>
+      <x:c r="X62" s="23" t="str"/>
+      <x:c r="Y62" s="23" t="str"/>
+      <x:c r="Z62" s="23" t="str"/>
+      <x:c r="AA62" s="24" t="str"/>
     </x:row>
     <x:row r="63" ht="60" customHeight="1">
       <x:c r="A63" s="3" t="str">
@@ -7397,6 +8553,12 @@
       <x:c r="U63" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
+      <x:c r="V63" s="23" t="str"/>
+      <x:c r="W63" s="23" t="str"/>
+      <x:c r="X63" s="23" t="str"/>
+      <x:c r="Y63" s="23" t="str"/>
+      <x:c r="Z63" s="23" t="str"/>
+      <x:c r="AA63" s="24" t="str"/>
     </x:row>
     <x:row r="64" ht="60" customHeight="1">
       <x:c r="A64" s="3" t="str">
@@ -7452,8 +8614,14 @@
       <x:c r="U64" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="65" ht="60" customHeight="1">
+      <x:c r="V64" s="23" t="str"/>
+      <x:c r="W64" s="23" t="str"/>
+      <x:c r="X64" s="23" t="str"/>
+      <x:c r="Y64" s="23" t="str"/>
+      <x:c r="Z64" s="23" t="str"/>
+      <x:c r="AA64" s="24" t="str"/>
+    </x:row>
+    <x:row r="65" ht="164" customHeight="1">
       <x:c r="A65" s="3" t="str">
         <x:v>CSE 351</x:v>
       </x:c>
@@ -7515,8 +8683,37 @@
       <x:c r="U65" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="66" ht="60" customHeight="1">
+      <x:c r="V65" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W65" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X65" s="23" t="str">
+        <x:v>Joint offering: CSE 351 C (SLN 12932). Not a lecture/quiz pairing approval
+Majors only: C SCI, CMP E</x:v>
+      </x:c>
+      <x:c r="Y65" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Offered jointly with CSE 351 C
+C SCI,CMP E majors only
+--
+CSE MAJORS ONLY
+--
+--
+FINAL EXAM TENTATIVELY PLANNED FOR
+MARCH 17, 1230-220PM
+--</x:v>
+      </x:c>
+      <x:c r="Z65" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12921</x:v>
+      </x:c>
+      <x:c r="AA65" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="80" customHeight="1">
       <x:c r="A66" s="3" t="str">
         <x:v>CSE 351</x:v>
       </x:c>
@@ -7572,8 +8769,29 @@
       <x:c r="U66" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="67" ht="60" customHeight="1">
+      <x:c r="V66" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W66" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X66" s="23" t="str">
+        <x:v>Joint offering: CSE 351 CA (SLN 12933). Not a lecture/quiz pairing approval</x:v>
+      </x:c>
+      <x:c r="Y66" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Offered jointly with CSE 351 CA
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z66" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12922</x:v>
+      </x:c>
+      <x:c r="AA66" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="80" customHeight="1">
       <x:c r="A67" s="3" t="str">
         <x:v>CSE 351</x:v>
       </x:c>
@@ -7629,8 +8847,29 @@
       <x:c r="U67" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="68" ht="60" customHeight="1">
+      <x:c r="V67" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W67" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X67" s="23" t="str">
+        <x:v>Joint offering: CSE 351 CB (SLN 12934). Not a lecture/quiz pairing approval</x:v>
+      </x:c>
+      <x:c r="Y67" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Offered jointly with CSE 351 CB
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z67" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12923</x:v>
+      </x:c>
+      <x:c r="AA67" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="80" customHeight="1">
       <x:c r="A68" s="3" t="str">
         <x:v>CSE 351</x:v>
       </x:c>
@@ -7686,8 +8925,29 @@
       <x:c r="U68" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="69" ht="60" customHeight="1">
+      <x:c r="V68" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W68" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X68" s="23" t="str">
+        <x:v>Joint offering: CSE 351 CC (SLN 12935). Not a lecture/quiz pairing approval</x:v>
+      </x:c>
+      <x:c r="Y68" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Offered jointly with CSE 351 CC
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z68" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12924</x:v>
+      </x:c>
+      <x:c r="AA68" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="80" customHeight="1">
       <x:c r="A69" s="3" t="str">
         <x:v>CSE 351</x:v>
       </x:c>
@@ -7743,8 +9003,29 @@
       <x:c r="U69" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="70" ht="60" customHeight="1">
+      <x:c r="V69" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W69" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X69" s="23" t="str">
+        <x:v>Joint offering: CSE 351 CD (SLN 12936). Not a lecture/quiz pairing approval</x:v>
+      </x:c>
+      <x:c r="Y69" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Offered jointly with CSE 351 CD
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z69" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12925</x:v>
+      </x:c>
+      <x:c r="AA69" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="80" customHeight="1">
       <x:c r="A70" s="3" t="str">
         <x:v>CSE 351</x:v>
       </x:c>
@@ -7800,8 +9081,29 @@
       <x:c r="U70" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="71" ht="60" customHeight="1">
+      <x:c r="V70" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W70" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X70" s="23" t="str">
+        <x:v>Joint offering: CSE 351 CE (SLN 12937). Not a lecture/quiz pairing approval</x:v>
+      </x:c>
+      <x:c r="Y70" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Offered jointly with CSE 351 CE
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z70" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12926</x:v>
+      </x:c>
+      <x:c r="AA70" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="150" customHeight="1">
       <x:c r="A71" s="3" t="str">
         <x:v>CSE 351</x:v>
       </x:c>
@@ -7863,8 +9165,36 @@
       <x:c r="U71" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="72" ht="60" customHeight="1">
+      <x:c r="V71" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W71" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X71" s="23" t="str">
+        <x:v>Joint offering: CSE 351 D (SLN 12938). Not a lecture/quiz pairing approval
+Majors only: C SCI, CMP E</x:v>
+      </x:c>
+      <x:c r="Y71" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Offered jointly with CSE 351 D
+C SCI,CMP E majors only
+--
+CSE MAJORS ONLY
+--
+FINAL EXAM TENTATIVELY PLANNED FOR
+MARCH 17, 1230-220PM
+--</x:v>
+      </x:c>
+      <x:c r="Z71" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12927</x:v>
+      </x:c>
+      <x:c r="AA71" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="80" customHeight="1">
       <x:c r="A72" s="3" t="str">
         <x:v>CSE 351</x:v>
       </x:c>
@@ -7920,8 +9250,29 @@
       <x:c r="U72" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="73" ht="60" customHeight="1">
+      <x:c r="V72" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W72" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X72" s="23" t="str">
+        <x:v>Joint offering: CSE 351 DA (SLN 12939). Not a lecture/quiz pairing approval</x:v>
+      </x:c>
+      <x:c r="Y72" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Offered jointly with CSE 351 DA
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z72" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12928</x:v>
+      </x:c>
+      <x:c r="AA72" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="80" customHeight="1">
       <x:c r="A73" s="3" t="str">
         <x:v>CSE 351</x:v>
       </x:c>
@@ -7977,8 +9328,29 @@
       <x:c r="U73" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="74" ht="60" customHeight="1">
+      <x:c r="V73" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W73" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X73" s="23" t="str">
+        <x:v>Joint offering: CSE 351 DB (SLN 12940). Not a lecture/quiz pairing approval</x:v>
+      </x:c>
+      <x:c r="Y73" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Offered jointly with CSE 351 DB
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z73" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12929</x:v>
+      </x:c>
+      <x:c r="AA73" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="80" customHeight="1">
       <x:c r="A74" s="3" t="str">
         <x:v>CSE 351</x:v>
       </x:c>
@@ -8034,8 +9406,29 @@
       <x:c r="U74" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="75" ht="60" customHeight="1">
+      <x:c r="V74" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W74" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X74" s="23" t="str">
+        <x:v>Joint offering: CSE 351 DC (SLN 12941). Not a lecture/quiz pairing approval</x:v>
+      </x:c>
+      <x:c r="Y74" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Offered jointly with CSE 351 DC
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z74" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12930</x:v>
+      </x:c>
+      <x:c r="AA74" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75" ht="80" customHeight="1">
       <x:c r="A75" s="3" t="str">
         <x:v>CSE 351</x:v>
       </x:c>
@@ -8091,8 +9484,29 @@
       <x:c r="U75" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="76" ht="60" customHeight="1">
+      <x:c r="V75" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W75" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X75" s="23" t="str">
+        <x:v>Joint offering: CSE 351 DD (SLN 12942). Not a lecture/quiz pairing approval</x:v>
+      </x:c>
+      <x:c r="Y75" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Offered jointly with CSE 351 DD
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z75" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12931</x:v>
+      </x:c>
+      <x:c r="AA75" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76" ht="150" customHeight="1">
       <x:c r="A76" s="3" t="str">
         <x:v>CSE 351</x:v>
       </x:c>
@@ -8154,8 +9568,36 @@
       <x:c r="U76" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="77" ht="60" customHeight="1">
+      <x:c r="V76" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W76" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X76" s="23" t="str">
+        <x:v>Joint offering: CSE 351 A (SLN 12921). Not a lecture/quiz pairing approval
+Majors only: E E, ECENG, ECE</x:v>
+      </x:c>
+      <x:c r="Y76" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Offered jointly with CSE 351 A
+E E,ECENG,ECE majors only
+--
+ECE MAJORS ONLY
+--
+FINAL EXAM TENTATIVELY PLANNED FOR
+MARCH 17, 1230-220PM
+--</x:v>
+      </x:c>
+      <x:c r="Z76" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12932</x:v>
+      </x:c>
+      <x:c r="AA76" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77" ht="80" customHeight="1">
       <x:c r="A77" s="3" t="str">
         <x:v>CSE 351</x:v>
       </x:c>
@@ -8211,8 +9653,29 @@
       <x:c r="U77" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="78" ht="60" customHeight="1">
+      <x:c r="V77" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W77" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X77" s="23" t="str">
+        <x:v>Joint offering: CSE 351 AA (SLN 12922). Not a lecture/quiz pairing approval</x:v>
+      </x:c>
+      <x:c r="Y77" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Offered jointly with CSE 351 AA
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z77" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12933</x:v>
+      </x:c>
+      <x:c r="AA77" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78" ht="80" customHeight="1">
       <x:c r="A78" s="3" t="str">
         <x:v>CSE 351</x:v>
       </x:c>
@@ -8268,8 +9731,29 @@
       <x:c r="U78" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="79" ht="60" customHeight="1">
+      <x:c r="V78" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W78" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X78" s="23" t="str">
+        <x:v>Joint offering: CSE 351 AB (SLN 12923). Not a lecture/quiz pairing approval</x:v>
+      </x:c>
+      <x:c r="Y78" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Offered jointly with CSE 351 AB
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z78" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12934</x:v>
+      </x:c>
+      <x:c r="AA78" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79" ht="80" customHeight="1">
       <x:c r="A79" s="3" t="str">
         <x:v>CSE 351</x:v>
       </x:c>
@@ -8325,8 +9809,29 @@
       <x:c r="U79" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="80" ht="60" customHeight="1">
+      <x:c r="V79" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W79" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X79" s="23" t="str">
+        <x:v>Joint offering: CSE 351 AC (SLN 12924). Not a lecture/quiz pairing approval</x:v>
+      </x:c>
+      <x:c r="Y79" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Offered jointly with CSE 351 AC
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z79" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12935</x:v>
+      </x:c>
+      <x:c r="AA79" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80" ht="80" customHeight="1">
       <x:c r="A80" s="3" t="str">
         <x:v>CSE 351</x:v>
       </x:c>
@@ -8382,8 +9887,29 @@
       <x:c r="U80" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="81" ht="60" customHeight="1">
+      <x:c r="V80" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W80" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X80" s="23" t="str">
+        <x:v>Joint offering: CSE 351 AD (SLN 12925). Not a lecture/quiz pairing approval</x:v>
+      </x:c>
+      <x:c r="Y80" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Offered jointly with CSE 351 AD
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z80" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12936</x:v>
+      </x:c>
+      <x:c r="AA80" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81" ht="80" customHeight="1">
       <x:c r="A81" s="3" t="str">
         <x:v>CSE 351</x:v>
       </x:c>
@@ -8439,8 +9965,29 @@
       <x:c r="U81" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="82" ht="60" customHeight="1">
+      <x:c r="V81" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W81" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X81" s="23" t="str">
+        <x:v>Joint offering: CSE 351 AE (SLN 12926). Not a lecture/quiz pairing approval</x:v>
+      </x:c>
+      <x:c r="Y81" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Offered jointly with CSE 351 AE
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z81" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12937</x:v>
+      </x:c>
+      <x:c r="AA81" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82" ht="150" customHeight="1">
       <x:c r="A82" s="3" t="str">
         <x:v>CSE 351</x:v>
       </x:c>
@@ -8502,8 +10049,36 @@
       <x:c r="U82" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="83" ht="60" customHeight="1">
+      <x:c r="V82" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W82" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X82" s="23" t="str">
+        <x:v>Joint offering: CSE 351 B (SLN 12927). Not a lecture/quiz pairing approval
+Majors only: E E, ECE, ECENG</x:v>
+      </x:c>
+      <x:c r="Y82" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Offered jointly with CSE 351 B
+E E,ECE,ECENG majors only
+--
+ECE MAJORS ONLY
+--
+FINAL EXAM TENTATIVELY PLANNED FOR
+MARCH 17, 1230-220PM
+--</x:v>
+      </x:c>
+      <x:c r="Z82" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12938</x:v>
+      </x:c>
+      <x:c r="AA82" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83" ht="80" customHeight="1">
       <x:c r="A83" s="3" t="str">
         <x:v>CSE 351</x:v>
       </x:c>
@@ -8559,8 +10134,29 @@
       <x:c r="U83" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="84" ht="60" customHeight="1">
+      <x:c r="V83" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W83" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X83" s="23" t="str">
+        <x:v>Joint offering: CSE 351 BA (SLN 12928). Not a lecture/quiz pairing approval</x:v>
+      </x:c>
+      <x:c r="Y83" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Offered jointly with CSE 351 BA
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z83" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12939</x:v>
+      </x:c>
+      <x:c r="AA83" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84" ht="80" customHeight="1">
       <x:c r="A84" s="3" t="str">
         <x:v>CSE 351</x:v>
       </x:c>
@@ -8616,8 +10212,29 @@
       <x:c r="U84" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="85" ht="60" customHeight="1">
+      <x:c r="V84" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W84" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X84" s="23" t="str">
+        <x:v>Joint offering: CSE 351 BB (SLN 12929). Not a lecture/quiz pairing approval</x:v>
+      </x:c>
+      <x:c r="Y84" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Offered jointly with CSE 351 BB
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z84" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12940</x:v>
+      </x:c>
+      <x:c r="AA84" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85" ht="80" customHeight="1">
       <x:c r="A85" s="3" t="str">
         <x:v>CSE 351</x:v>
       </x:c>
@@ -8673,8 +10290,29 @@
       <x:c r="U85" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="86" ht="60" customHeight="1">
+      <x:c r="V85" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W85" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X85" s="23" t="str">
+        <x:v>Joint offering: CSE 351 BC (SLN 12930). Not a lecture/quiz pairing approval</x:v>
+      </x:c>
+      <x:c r="Y85" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Offered jointly with CSE 351 BC
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z85" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12941</x:v>
+      </x:c>
+      <x:c r="AA85" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86" ht="80" customHeight="1">
       <x:c r="A86" s="3" t="str">
         <x:v>CSE 351</x:v>
       </x:c>
@@ -8730,8 +10368,29 @@
       <x:c r="U86" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="87" ht="60" customHeight="1">
+      <x:c r="V86" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W86" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X86" s="23" t="str">
+        <x:v>Joint offering: CSE 351 BD (SLN 12931). Not a lecture/quiz pairing approval</x:v>
+      </x:c>
+      <x:c r="Y86" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Offered jointly with CSE 351 BD
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z86" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12942</x:v>
+      </x:c>
+      <x:c r="AA86" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87" ht="80" customHeight="1">
       <x:c r="A87" s="3" t="str">
         <x:v>CSE 373</x:v>
       </x:c>
@@ -8791,8 +10450,29 @@
       <x:c r="U87" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="88" ht="60" customHeight="1">
+      <x:c r="V87" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W87" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X87" s="23" t="str">
+        <x:v>Excluded majors: C SCI, CMP E</x:v>
+      </x:c>
+      <x:c r="Y87" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+No C SCI,CMP E majors
+CSE NON-MAJOR COURSE</x:v>
+      </x:c>
+      <x:c r="Z87" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12945</x:v>
+      </x:c>
+      <x:c r="AA87" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88" ht="80" customHeight="1">
       <x:c r="A88" s="3" t="str">
         <x:v>CSE 373</x:v>
       </x:c>
@@ -8846,8 +10526,28 @@
       <x:c r="U88" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="89" ht="60" customHeight="1">
+      <x:c r="V88" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W88" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X88" s="23" t="str">
+        <x:v>No additional structured restriction in captured Notes. Full eligibility remains unknown.</x:v>
+      </x:c>
+      <x:c r="Y88" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z88" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12946</x:v>
+      </x:c>
+      <x:c r="AA88" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89" ht="80" customHeight="1">
       <x:c r="A89" s="3" t="str">
         <x:v>CSE 373</x:v>
       </x:c>
@@ -8901,8 +10601,28 @@
       <x:c r="U89" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="90" ht="60" customHeight="1">
+      <x:c r="V89" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W89" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X89" s="23" t="str">
+        <x:v>No additional structured restriction in captured Notes. Full eligibility remains unknown.</x:v>
+      </x:c>
+      <x:c r="Y89" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z89" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12947</x:v>
+      </x:c>
+      <x:c r="AA89" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90" ht="80" customHeight="1">
       <x:c r="A90" s="3" t="str">
         <x:v>CSE 373</x:v>
       </x:c>
@@ -8956,8 +10676,28 @@
       <x:c r="U90" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="91" ht="60" customHeight="1">
+      <x:c r="V90" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W90" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X90" s="23" t="str">
+        <x:v>No additional structured restriction in captured Notes. Full eligibility remains unknown.</x:v>
+      </x:c>
+      <x:c r="Y90" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z90" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12948</x:v>
+      </x:c>
+      <x:c r="AA90" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91" ht="80" customHeight="1">
       <x:c r="A91" s="3" t="str">
         <x:v>CSE 373</x:v>
       </x:c>
@@ -9011,8 +10751,28 @@
       <x:c r="U91" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="92" ht="60" customHeight="1">
+      <x:c r="V91" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W91" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X91" s="23" t="str">
+        <x:v>No additional structured restriction in captured Notes. Full eligibility remains unknown.</x:v>
+      </x:c>
+      <x:c r="Y91" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z91" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12949</x:v>
+      </x:c>
+      <x:c r="AA91" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92" ht="80" customHeight="1">
       <x:c r="A92" s="3" t="str">
         <x:v>CSE 373</x:v>
       </x:c>
@@ -9066,8 +10826,28 @@
       <x:c r="U92" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="93" ht="60" customHeight="1">
+      <x:c r="V92" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W92" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X92" s="23" t="str">
+        <x:v>No additional structured restriction in captured Notes. Full eligibility remains unknown.</x:v>
+      </x:c>
+      <x:c r="Y92" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z92" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12950</x:v>
+      </x:c>
+      <x:c r="AA92" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93" ht="80" customHeight="1">
       <x:c r="A93" s="3" t="str">
         <x:v>CSE 373</x:v>
       </x:c>
@@ -9121,8 +10901,28 @@
       <x:c r="U93" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="94" ht="60" customHeight="1">
+      <x:c r="V93" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W93" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X93" s="23" t="str">
+        <x:v>No additional structured restriction in captured Notes. Full eligibility remains unknown.</x:v>
+      </x:c>
+      <x:c r="Y93" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z93" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12951</x:v>
+      </x:c>
+      <x:c r="AA93" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94" ht="80" customHeight="1">
       <x:c r="A94" s="3" t="str">
         <x:v>CSE 373</x:v>
       </x:c>
@@ -9176,8 +10976,28 @@
       <x:c r="U94" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="95" ht="60" customHeight="1">
+      <x:c r="V94" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W94" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X94" s="23" t="str">
+        <x:v>No additional structured restriction in captured Notes. Full eligibility remains unknown.</x:v>
+      </x:c>
+      <x:c r="Y94" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section</x:v>
+      </x:c>
+      <x:c r="Z94" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12952</x:v>
+      </x:c>
+      <x:c r="AA94" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95" ht="122" customHeight="1">
       <x:c r="A95" s="3" t="str">
         <x:v>CSE 373</x:v>
       </x:c>
@@ -9235,8 +11055,34 @@
       <x:c r="U95" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="96" ht="60" customHeight="1">
+      <x:c r="V95" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W95" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X95" s="23" t="str">
+        <x:v>Add code required
+Tentative section. Exclude by default</x:v>
+      </x:c>
+      <x:c r="Y95" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section
+Add Code required
+--
+TENTATIVE
+SECTION WILL OPEN IF NEEDED
+--</x:v>
+      </x:c>
+      <x:c r="Z95" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12953</x:v>
+      </x:c>
+      <x:c r="AA95" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96" ht="122" customHeight="1">
       <x:c r="A96" s="3" t="str">
         <x:v>CSE 373</x:v>
       </x:c>
@@ -9294,8 +11140,34 @@
       <x:c r="U96" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="97" ht="60" customHeight="1">
+      <x:c r="V96" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W96" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X96" s="23" t="str">
+        <x:v>Add code required
+Tentative section. Exclude by default</x:v>
+      </x:c>
+      <x:c r="Y96" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section
+Add Code required
+--
+TENTATIVE
+SECTION WILL OPEN IF NEEDED
+--</x:v>
+      </x:c>
+      <x:c r="Z96" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12954</x:v>
+      </x:c>
+      <x:c r="AA96" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97" ht="122" customHeight="1">
       <x:c r="A97" s="3" t="str">
         <x:v>CSE 373</x:v>
       </x:c>
@@ -9353,6 +11225,32 @@
       <x:c r="U97" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
+      <x:c r="V97" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W97" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X97" s="23" t="str">
+        <x:v>Add code required
+Tentative section. Exclude by default</x:v>
+      </x:c>
+      <x:c r="Y97" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Quiz Section
+Add Code required
+--
+TENTATIVE
+SECTION WILL OPEN IF NEEDED
+--</x:v>
+      </x:c>
+      <x:c r="Z97" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=12955</x:v>
+      </x:c>
+      <x:c r="AA97" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="98" ht="60" customHeight="1">
       <x:c r="A98" s="3" t="str">
@@ -9418,6 +11316,12 @@
       <x:c r="U98" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
+      <x:c r="V98" s="23" t="str"/>
+      <x:c r="W98" s="23" t="str"/>
+      <x:c r="X98" s="23" t="str"/>
+      <x:c r="Y98" s="23" t="str"/>
+      <x:c r="Z98" s="23" t="str"/>
+      <x:c r="AA98" s="24" t="str"/>
     </x:row>
     <x:row r="99" ht="60" customHeight="1">
       <x:c r="A99" s="3" t="str">
@@ -9483,6 +11387,12 @@
       <x:c r="U99" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
+      <x:c r="V99" s="23" t="str"/>
+      <x:c r="W99" s="23" t="str"/>
+      <x:c r="X99" s="23" t="str"/>
+      <x:c r="Y99" s="23" t="str"/>
+      <x:c r="Z99" s="23" t="str"/>
+      <x:c r="AA99" s="24" t="str"/>
     </x:row>
     <x:row r="100" ht="60" customHeight="1">
       <x:c r="A100" s="3" t="str">
@@ -9544,6 +11454,12 @@
       <x:c r="U100" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
+      <x:c r="V100" s="23" t="str"/>
+      <x:c r="W100" s="23" t="str"/>
+      <x:c r="X100" s="23" t="str"/>
+      <x:c r="Y100" s="23" t="str"/>
+      <x:c r="Z100" s="23" t="str"/>
+      <x:c r="AA100" s="24" t="str"/>
     </x:row>
     <x:row r="101" ht="60" customHeight="1">
       <x:c r="A101" s="3" t="str">
@@ -9599,6 +11515,12 @@
       <x:c r="U101" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
+      <x:c r="V101" s="23" t="str"/>
+      <x:c r="W101" s="23" t="str"/>
+      <x:c r="X101" s="23" t="str"/>
+      <x:c r="Y101" s="23" t="str"/>
+      <x:c r="Z101" s="23" t="str"/>
+      <x:c r="AA101" s="24" t="str"/>
     </x:row>
     <x:row r="102" ht="60" customHeight="1">
       <x:c r="A102" s="3" t="str">
@@ -9654,6 +11576,12 @@
       <x:c r="U102" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
+      <x:c r="V102" s="23" t="str"/>
+      <x:c r="W102" s="23" t="str"/>
+      <x:c r="X102" s="23" t="str"/>
+      <x:c r="Y102" s="23" t="str"/>
+      <x:c r="Z102" s="23" t="str"/>
+      <x:c r="AA102" s="24" t="str"/>
     </x:row>
     <x:row r="103" ht="60" customHeight="1">
       <x:c r="A103" s="3" t="str">
@@ -9709,6 +11637,12 @@
       <x:c r="U103" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
+      <x:c r="V103" s="23" t="str"/>
+      <x:c r="W103" s="23" t="str"/>
+      <x:c r="X103" s="23" t="str"/>
+      <x:c r="Y103" s="23" t="str"/>
+      <x:c r="Z103" s="23" t="str"/>
+      <x:c r="AA103" s="24" t="str"/>
     </x:row>
     <x:row r="104" ht="60" customHeight="1">
       <x:c r="A104" s="3" t="str">
@@ -9764,6 +11698,12 @@
       <x:c r="U104" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
+      <x:c r="V104" s="23" t="str"/>
+      <x:c r="W104" s="23" t="str"/>
+      <x:c r="X104" s="23" t="str"/>
+      <x:c r="Y104" s="23" t="str"/>
+      <x:c r="Z104" s="23" t="str"/>
+      <x:c r="AA104" s="24" t="str"/>
     </x:row>
     <x:row r="105" ht="60" customHeight="1">
       <x:c r="A105" s="3" t="str">
@@ -9819,6 +11759,12 @@
       <x:c r="U105" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
+      <x:c r="V105" s="23" t="str"/>
+      <x:c r="W105" s="23" t="str"/>
+      <x:c r="X105" s="23" t="str"/>
+      <x:c r="Y105" s="23" t="str"/>
+      <x:c r="Z105" s="23" t="str"/>
+      <x:c r="AA105" s="24" t="str"/>
     </x:row>
     <x:row r="106" ht="60" customHeight="1">
       <x:c r="A106" s="3" t="str">
@@ -9874,8 +11820,14 @@
       <x:c r="U106" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="107" ht="60" customHeight="1">
+      <x:c r="V106" s="23" t="str"/>
+      <x:c r="W106" s="23" t="str"/>
+      <x:c r="X106" s="23" t="str"/>
+      <x:c r="Y106" s="23" t="str"/>
+      <x:c r="Z106" s="23" t="str"/>
+      <x:c r="AA106" s="24" t="str"/>
+    </x:row>
+    <x:row r="107" ht="80" customHeight="1">
       <x:c r="A107" s="3" t="str">
         <x:v>AMATH 301</x:v>
       </x:c>
@@ -9935,8 +11887,30 @@
       <x:c r="U107" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="108" ht="60" customHeight="1">
+      <x:c r="V107" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W107" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X107" s="23" t="str">
+        <x:v>Additional fee: USD 22</x:v>
+      </x:c>
+      <x:c r="Y107" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+$22 additional course fee req'd
+Fee purpose: Other
+PYTHON</x:v>
+      </x:c>
+      <x:c r="Z107" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=10211</x:v>
+      </x:c>
+      <x:c r="AA107" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108" ht="80" customHeight="1">
       <x:c r="A108" s="3" t="str">
         <x:v>AMATH 301</x:v>
       </x:c>
@@ -9996,8 +11970,30 @@
       <x:c r="U108" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="109" ht="60" customHeight="1">
+      <x:c r="V108" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W108" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X108" s="23" t="str">
+        <x:v>Additional fee: USD 22</x:v>
+      </x:c>
+      <x:c r="Y108" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+$22 additional course fee req'd
+Fee purpose: Other
+PYTHON</x:v>
+      </x:c>
+      <x:c r="Z108" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=10212</x:v>
+      </x:c>
+      <x:c r="AA108" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109" ht="80" customHeight="1">
       <x:c r="A109" s="3" t="str">
         <x:v>AMATH 301</x:v>
       </x:c>
@@ -10057,8 +12053,30 @@
       <x:c r="U109" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="110" ht="60" customHeight="1">
+      <x:c r="V109" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W109" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X109" s="23" t="str">
+        <x:v>Additional fee: USD 22</x:v>
+      </x:c>
+      <x:c r="Y109" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+$22 additional course fee req'd
+Fee purpose: Other
+PYTHON</x:v>
+      </x:c>
+      <x:c r="Z109" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=10213</x:v>
+      </x:c>
+      <x:c r="AA109" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110" ht="80" customHeight="1">
       <x:c r="A110" s="3" t="str">
         <x:v>AMATH 351</x:v>
       </x:c>
@@ -10118,8 +12136,30 @@
       <x:c r="U110" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="111" ht="60" customHeight="1">
+      <x:c r="V110" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W110" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X110" s="23" t="str">
+        <x:v>Majors only: AMATH, CFRM, ACMS. Period I only: 2026-11-05 through 2026-11-22 (inclusive)</x:v>
+      </x:c>
+      <x:c r="Y110" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+AMATH,CFRM,ACMS majors only Period 1 (11/5/2026-11/22/2026)
+ADD CODE POLICY:
+AMATH.WASHINGTON.EDU/ADVISING</x:v>
+      </x:c>
+      <x:c r="Z110" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=10215</x:v>
+      </x:c>
+      <x:c r="AA110" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111" ht="80" customHeight="1">
       <x:c r="A111" s="3" t="str">
         <x:v>AMATH 351</x:v>
       </x:c>
@@ -10179,8 +12219,30 @@
       <x:c r="U111" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="112" ht="60" customHeight="1">
+      <x:c r="V111" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W111" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X111" s="23" t="str">
+        <x:v>Majors only: AMATH, CFRM, ACMS. Period I only: 2026-11-05 through 2026-11-22 (inclusive)</x:v>
+      </x:c>
+      <x:c r="Y111" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+AMATH,CFRM,ACMS majors only Period 1 (11/5/2026-11/22/2026)
+ADD CODE POLICY:
+AMATH.WASHINGTON.EDU/ADVISING</x:v>
+      </x:c>
+      <x:c r="Z111" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=10216</x:v>
+      </x:c>
+      <x:c r="AA111" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="112" ht="94" customHeight="1">
       <x:c r="A112" s="3" t="str">
         <x:v>AMATH 352</x:v>
       </x:c>
@@ -10240,8 +12302,32 @@
       <x:c r="U112" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="113" ht="60" customHeight="1">
+      <x:c r="V112" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W112" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X112" s="23" t="str">
+        <x:v>Excluded student level: graduate
+Majors only: AMATH, CFRM, ACMS. Period I only: 2026-11-05 through 2026-11-22 (inclusive)</x:v>
+      </x:c>
+      <x:c r="Y112" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+No Grads
+AMATH,CFRM,ACMS majors only Period 1 (11/5/2026-11/22/2026)
+ADD CODE POLICY:
+AMATH.WASHINGTON.EDU/ADVISING</x:v>
+      </x:c>
+      <x:c r="Z112" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=10217</x:v>
+      </x:c>
+      <x:c r="AA112" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113" ht="94" customHeight="1">
       <x:c r="A113" s="3" t="str">
         <x:v>AMATH 352</x:v>
       </x:c>
@@ -10301,6 +12387,30 @@
       <x:c r="U113" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
+      <x:c r="V113" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W113" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X113" s="23" t="str">
+        <x:v>Excluded student level: graduate
+Majors only: AMATH, CFRM, ACMS. Period I only: 2026-11-05 through 2026-11-22 (inclusive)</x:v>
+      </x:c>
+      <x:c r="Y113" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+No Grads
+AMATH,CFRM,ACMS majors only Period 1 (11/5/2026-11/22/2026)
+ADD CODE POLICY:
+AMATH.WASHINGTON.EDU/ADVISING</x:v>
+      </x:c>
+      <x:c r="Z113" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=10218</x:v>
+      </x:c>
+      <x:c r="AA113" s="24" t="n">
+        <x:v>46312.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="114" ht="60" customHeight="1">
       <x:c r="A114" s="3" t="str">
@@ -10362,6 +12472,12 @@
       <x:c r="U114" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
+      <x:c r="V114" s="23" t="str"/>
+      <x:c r="W114" s="23" t="str"/>
+      <x:c r="X114" s="23" t="str"/>
+      <x:c r="Y114" s="23" t="str"/>
+      <x:c r="Z114" s="23" t="str"/>
+      <x:c r="AA114" s="24" t="str"/>
     </x:row>
     <x:row r="115" ht="60" customHeight="1">
       <x:c r="A115" s="3" t="str">
@@ -10423,8 +12539,14 @@
       <x:c r="U115" s="11" t="n">
         <x:v>46312.00208333333</x:v>
       </x:c>
-    </x:row>
-    <x:row r="116" ht="60" customHeight="1">
+      <x:c r="V115" s="23" t="str"/>
+      <x:c r="W115" s="23" t="str"/>
+      <x:c r="X115" s="23" t="str"/>
+      <x:c r="Y115" s="23" t="str"/>
+      <x:c r="Z115" s="23" t="str"/>
+      <x:c r="AA115" s="24" t="str"/>
+    </x:row>
+    <x:row r="116" ht="234" customHeight="1">
       <x:c r="A116" s="3" t="str">
         <x:v>AMATH 482</x:v>
       </x:c>
@@ -10483,6 +12605,42 @@
       </x:c>
       <x:c r="U116" s="11" t="n">
         <x:v>46312.00208333333</x:v>
+      </x:c>
+      <x:c r="V116" s="23" t="str">
+        <x:v>SLN_notes_read</x:v>
+      </x:c>
+      <x:c r="W116" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="X116" s="23" t="str">
+        <x:v>Waitlist applies only when registration is restricted by add code
+Excluded student level: graduate
+Majors only: AMATH, CFRM, ACMS. Period I only: 2026-11-05 through 2026-11-22 (inclusive)
+Registration subject to prerequisite cancellation</x:v>
+      </x:c>
+      <x:c r="Y116" s="23" t="str">
+        <x:v>Notes
+Check prerequisites
+Students who do not complete the prerequisites will be dropped from this course.
+No Grads
+AMATH,CFRM,ACMS majors only Period 1 (11/5/2026-11/22/2026)
+ADD CODE POLICY:
+AMATH.WASHINGTON.EDU/ADVISING
+ADD CODE WAITLIST:
+HTTPS://TINYURL.COM/YSW78KW2
+--
+IF COURSE REGISTRATION NOT
+RESTRICTED BY ADD CODE, WAITLIST
+WILL NOT BE USED.
+USE UW NOTIFY TO BE NOTIFIED OF
+SEAT AVAILABILITY AND ATTEMPT TO
+GAIN A SEAT.</x:v>
+      </x:c>
+      <x:c r="Z116" s="23" t="str">
+        <x:v>https://sdb.admin.uw.edu/timeschd/uwnetid/sln.asp?QTRYR=WIN+2027&amp;SLN=10222</x:v>
+      </x:c>
+      <x:c r="AA116" s="24" t="n">
+        <x:v>46312.5</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -10491,7 +12649,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38fcc6cfc491470b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0293708f8184225"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23293,7 +25451,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7df16314e97a4556"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9c731e535a843db"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>